<commit_message>
fix: lockfile issue during run
</commit_message>
<xml_diff>
--- a/TestData/UploadFiles/RequestEndPoint.xlsx
+++ b/TestData/UploadFiles/RequestEndPoint.xlsx
@@ -241,19 +241,16 @@
     <x:t>UpdatedAt</x:t>
   </x:si>
   <x:si>
-    <x:t>c00640ec-b743-4728-87d2-a39dc1309e5f</x:t>
+    <x:t>2026-10-08T11:23:04.8753507Z</x:t>
   </x:si>
   <x:si>
     <x:t/>
   </x:si>
   <x:si>
-    <x:t>2026-10-07T13:24:55.6248021Z</x:t>
-  </x:si>
-  <x:si>
     <x:t>9eb45736-827a-4751-9996-44088587006e</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-10-07T13:24:55.5406269Z</x:t>
+    <x:t>2026-10-08T11:23:04.7663825Z</x:t>
   </x:si>
   <x:si>
     <x:t>login</x:t>
@@ -265,16 +262,19 @@
     <x:t>200</x:t>
   </x:si>
   <x:si>
-    <x:t>{"access_token":"eyJhbGciOiJSUzI1NiIsImtpZCI6Ilg1ZVhrNHh5b2pORnVtMWtsMll0djhkbE5QNC1jNTdkTzZRR1RWQndhTmsiLCJ0eXAiOiJKV1QifQ.eyJhdWQiOiJjOTdhMGNjOC05MTIzLTQxMDgtYTljMS03ZDliZDJhNmI4YzAiLCJpc3MiOiJodHRwczovL3Rlc3Ryb3ZpY2FyZS5iMmNsb2dpbi5jb20vZjFmMGRmYzctM2EzYy00ZWMyLWIwOWMtNTRlZWQ4NGMyMGYxL3YyLjAvIiwiZXhwIjoxNzkxMzgzMDk0LCJuYmYiOjE3OTEzNzk0OTQsImlkcCI6IkxvY2FsQWNjb3VudCIsInN1YiI6IjA2M2E5YmY2LWNhOGItNGMxZi1hMGZiLTQ5OGY3YjIwMjBmYiIsImVtYWlscyI6WyJob3NwaXRhbEByb3ZpY2FyZS5jb20iXSwidGZwIjoiQjJDXzFfUk9QQ19UZXN0Iiwic2NwIjoiV2ViQ2xpZW50IiwiYXpwIjoiYzZhYmM1NjctM2Y0YS00YjEzLTg1OTMtNzY0YjIwOWExN2VhIiwidmVyIjoiMS4wIiwiaWF0IjoxNzkxMzc5NDk0fQ.eEZedSoLMDy5irTZLLi90u4TbkO-xz0Gm7JSrfQcIAKcim56L2bufxZaHKUmnrXja7zgQwkYM2_QRPKDT7e7x0EMapbDWOr1u0oCLA8r3rQVg8O99_vL0Hselbb9v0kleh-Pt-5u5MXxB5grL-zPYOkPQbqqM_8gK3RsR789U3MtuJ4T4r09FhlLAVRM0qtkdZPHIq_aGXiGOQynch7Z9Eo6qjDSSZz7bG_rP7-wxXQ1tz50QvW3SbVpjKJLbBls8QRti6AXRFW38p24yagBjhUnOVeFhsN7-u7tJ7oy4FTtDmZsfSYnptGG0Y_IOUAoepyFVfReJITxxn_Ba221nA","token_type":"Bearer","expires_in":"3600"}</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2026-10-07T13:24:54.6056362Z</x:t>
-  </x:si>
-  <x:si>
-    <x:t>{"MemberId":"9eb45736-827a-4751-9996-44088587006e","FirstName":"Arizona","LastName":"Rovicare ","UserName":"hospital@rovicare.com","EmailId":"hospital@rovicare.com","BusinessUnitId":"677920c1-831f-11ea-bd7d-04d9f5ab62dc","CompanyBusinessUnitId":"677920c1-831f-11ea-bd7d-04d9f5ab62dc","BusinessUnitName":"Arizona State Hospital","BusinessUnitType":"Provider","AssignedSettings":{"ReferralVisibilityInHrs":120,"ExtendedReferralVisibilityInHrs":192,"RatingReminderInDays":2,"ReferralViewDelayInMins":30,"IsEnableOrphanReferral":true,"IsEnable2StepAppointment":false,"AllowMemberAssigntoReferralForSendReferral":true,"AllowMemberViewAllReferralForSendReferral":true,"AllowMemberAssigntoReferralForReceiveReferral":false,"AllowMemberViewAllReferralForReceiveReferral":true,"DefaultHealthFacilityRating":2,"DefaultMedicareRating":4,"ReferralWithPatientPreferenceNote":null,"SearchAreaBy":"County","MaxSavedSearchAllowed":500,"IsContractSearched":false,"IsFaxReferralActive":true,"IsEmailReferralActive":true,"HadReferralWithAdvanceNotice":true,"WorkStartTime":null,"WorkEndTime":null,"MaxNumberOfOrganizationMembers":500,"MaxNumberOfImagesUploaded":10,"MaxSizeOfImagesUploadedInMB":50,"DurationOfHistoricalRecordsInDays":120,"LastSynOn":"2023-11-22T12:45:57.1111937Z","DefaultProviderType":null,"PatientVisibilityDays":30,"ConfirmReferralVisibilityInHrs":1.0,"LoginMethod":"Rovicare","DefaultFilter":"Medical","ShowInsurance":"Outgoing","IsTwelveTimeFormat":false,"ReceiveReferralDeliveryMode":"EFS","SendReferralToMemberViaFax":false,"EmrType":"Rovicare","EditRecordImportPatient":false,"AddRecordImportPatient":false,"OverrideRecordImportPatient":false,"AutomaticOverrideRecordImportPatient":true,"IsFullCapacity":true,"AcceptReferral":true,"IndicateToOrigin":true,"InpatientReferralActive":null,"OutpatientReferralActive":null,"PreAuthorizationRequired":false,"SharePatientRecord":false,"UpdateReferralResponse":true,"AutomaticallySharePatientRecord":false,"TentativeAcceptPatient":false,"ShowAverageResponseRate":true,"ResponseRateBusinessunitIds":"","DestinationCaseManagerConfig":"Email,Name,WorkNumber","CaseManagerDetailsConfig":"PhoneNumber,Email","DefaultShortlistPaginationCount":"50","DelayedClinicalRecordDays":null,"FaxNumberToSendCocDocument":null,"FollowUpRemovalTimeInMinutes":43200,"CocDocumentRequiringInsuranceList":[],"FollowUp7DayReminderTimeInMinute":10080,"FollowUp30DayReminderTimeInMinute":43200,"InpatientVisitReminderTimeInMinute":1440,"HiCommNotificationReminderInMinute":1440,"HiCommIPVDueDateOffsetDays":7,"CocDocumentReminderTimeInMinute":4320,"ShowAhcccsInfo":false,"UpdateCampus":false,"HiCommPatientReadmitIntervalInDays":30,"LocalTimeZoneId":null,"AssignPatientTagToHiCoM":null,"TeamAssignmentNotification":true,"WorkingDays":[],"Insurance":[],"CareRequirement":[],"ProviderType":[],"ServiceSetting":[],"SpecialProgram":[],"AgeGroup":[],"GenderType":[],"FacilityType":[],"AppointmentStatus":[],"FollowUpStatus":[],"DefaultRoute":null,"ConfigurableLogo":null,"Theme":null,"EnableDmeNotification":false,"WorkspaceConfigurations":[]},"DmeSettings":{"HcpNotificationMode":null,"EnableWoundCareQuantity":false,"EnableHhaCosmetics":false,"AllowShipToClinicianHome":false,"ShowEpisodeNumber":false},"EMRSetting":"{\"emrType\":\"Rovicare\",\"organizationName\":\"string\",\"organizationId\":\"string\",\"facilityId\":\"string\",\"AdvancedMdProgressNoteDateChanged\":\"string\",\"facilityUTCOffsetValue\":0.0,\"facilityAddress\":{\"streetAddress\":\"string\",\"city\":\"string\",\"state\":\"string\",\"zipcode\":\"string\"},\"providerType\":\"string\",\"facilityContact\":\"string\",\"healthCareResources\":{\"AllergyIntolerances\":true,\"Conditions\":true,\"Coverage\":true,\"DiagnosticReports\":true,\"Immunizations\":true,\"Medications\":true,\"ProgressNotes\":true,\"EmergencyContacts\":true,\"CarePlans\":true},\"MedicalRecordAccessLevel\":\"string\",\"HieFileInfo\":{\"BlobPathList\":[\"string\"],\"FileDirectoryFromUser\":\"string\",\"AddPatientIfNotExists\":true},\"siteId\":\"string\",\"fTPClientSettingModel\":{\"Host\":\"string\",\"Port\":0,\"UserName\":\"string\",\"Password\":\"string\",\"FileLocation\":\"string\",\"FileType\":\"string\"},\"EntityUpdates\":[{\"Entity\":\"string\",\"EntityLastUpdateTime\":\"2026-02-16T13:09:58.447Z\"}],\"EntityMetaData\":[{\"Entity\":\"string\",\"SearchParamters\":[{\"Key\":\"string\",\"Value\":\"string\"}]}]}","ServiceArea":"ZipCode","RoleName":"Organization Admin","HasAcceptedLicense":true,"AssignedFeatures":["NotificationFeature","ReceiveReferral","AppointmentDashboard","MobileApplication","SendReferral","ReceiveMedicalRecords","PreferredProviderList","Annotation","ShareCommandCenter","SurveyModule","CreateDMEOrder","ImportPatientByExcelsheet","SentReferralViaEmail","PendingServiceInitiationReminder","AddToPatientList","ShowCCRReport","GlobalChat","AdmitHistory","RecordReferral","PartialReferralConfirmation","AutoForwardChat","SentReferralViaFax","ShowReports","ShowCLRAReport","ReferralHistoryDashboard","AutomatedOriginStarRating","ShareReferrals","TagFeature","ShareMedicalRecords","LiveChat","PreferredProviderAvailability","CommandCenter","RecordReferralForOrigin","PendingReferralResponseReminder"],"BusinessUnitMemberId":"5b1a54d8-fd19-49f8-bb2e-fce04aa8b79e","PermissionList":["AcceptOrder","AddAppointment","AddAppointmentSlot","AddOrder","AddOrganization","AddOrganizationMember","AddPatient","AddPatientToCommandCenter","AddPreferredProvider","AddReferral","AddTag","AdminViewReports","AssignMember","AutoSyncOnAction","AutoSyncOnReferral","BulkActionForCommandCenter","CancelOrder","CancelReferral","CompulsaryServicesAndSpecialProgram","ConfirmPartialReferral","DeleteAppointment","DeleteAppointmentSlot","DeleteOrganizationMember","DeletePatient","DeletePreferredProvider","DeleteTag","DisableAutoConfirmReferral","DisableReferral","DisableReferralForServices","EditAppointment","EditAppointmentSlot","EditOrder","EditOrganization","EditOrganizationMember","EditPatient","EditPreferredProvider","EditReferral","EditTag","EnableMedicareRating","FaceSheetInMedicalRecords","GlobalChat","ImportPatientByCCDA","ImportPatientByExcelSheet","ImportPatientByFaceSheet","InsuranceProvider","LiveChat","ManageAllOrganization","ManageCompulsoryInsuranceForPatient","ManageCompulsoryServicesAndSpecialProgram","ManageOrganization","MemberAssignedToReferralForReceiveReferral","MessageBoard","MobileApplication","MovePatientToFollowUp","Notes","Notification","OnCallSupport","Order.Bulk.Download","Order.Bulk.Upload","Order.Bulk.View","Order.Document.Download","Order.Sign.Bypass","Order.Sign.OnBehalf","Order.Sign.Remind","Order.Workflow.Decline","Order.Workflow.Disposition","Order.Workflow.TakeOwnership","PatientPreference","PendingReferralsNotification","Prescriber.Search","ProvideRejectionReasonForReferral","ReceiveMedicalRecords","ReceiveReferral","ReceiveReferralSetting","ReferOrder","ReferralReport","ReferralTimeline","RejectOrder","RemovePatientFromCommandCenter","ResendReferral","ResponseReferral","ScheduleTransport","SendMedicalRecords","SendReferral","ShareCommandCenter","ShareMedicalRecords","ShareReferrals","ShareReferralsWithPreferredProviders","ShipOrder","ShowSpecialProgramNeeded","SuperAdmin","Track","UpdatePatientTask","UploadMedicalRecord","ViewAndManageCustomWorkspace","ViewAppointment","ViewAppointmentSlot","ViewMedicalRecord","ViewOrder","ViewOrganization","ViewOrganizationMember","ViewPatient","ViewPreferredProvider","ViewReferral","ViewReferralHistory","ViewTag"],"CacheId":"c00640ec-b743-4728-87d2-a39dc1309e5f","AcceptedPolicyIds":[],"LoginError":[],"HasPowerBiReportAccess":false}</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2026-10-07T13:24:55.5288357Z</x:t>
+    <x:t>{"access_token":"eyJhbGciOiJSUzI1NiIsImtpZCI6Ilg1ZVhrNHh5b2pORnVtMWtsMll0djhkbE5QNC1jNTdkTzZRR1RWQndhTmsiLCJ0eXAiOiJKV1QifQ.eyJhdWQiOiJjOTdhMGNjOC05MTIzLTQxMDgtYTljMS03ZDliZDJhNmI4YzAiLCJpc3MiOiJodHRwczovL3Rlc3Ryb3ZpY2FyZS5iMmNsb2dpbi5jb20vZjFmMGRmYzctM2EzYy00ZWMyLWIwOWMtNTRlZWQ4NGMyMGYxL3YyLjAvIiwiZXhwIjoxNzkxNDYyMTgzLCJuYmYiOjE3OTE0NTg1ODMsImlkcCI6IkxvY2FsQWNjb3VudCIsInN1YiI6IjA2M2E5YmY2LWNhOGItNGMxZi1hMGZiLTQ5OGY3YjIwMjBmYiIsImVtYWlscyI6WyJob3NwaXRhbEByb3ZpY2FyZS5jb20iXSwidGZwIjoiQjJDXzFfUk9QQ19UZXN0Iiwic2NwIjoiV2ViQ2xpZW50IiwiYXpwIjoiYzZhYmM1NjctM2Y0YS00YjEzLTg1OTMtNzY0YjIwOWExN2VhIiwidmVyIjoiMS4wIiwiaWF0IjoxNzkxNDU4NTgzfQ.KsWfqUI-r8TUyPoqLZoM3JXtkA-NCfAsyc3SWzlRXtIKe7XvINDNtutvcVWn03WBgmkPpwF8p5ofU3ACEuwNVnZuOaA_9Z3lI1-E1dVgVkFa55t4dxJKDqblmF9wrhlb1k6EdXOLULMyLElYY7Ac_L1tMoNr3wK4UxbXsY0pQMDnZW7BG1qOLZxyhvlmgUVMxkZQHTCUKUsZsEcNEf8EcDUKly-CO2g6dCOWIX_EpYuk5BtwLvHsVwcot9HJRelaq9fj-x6pjWm5fI6hF6TcRhYqGl123OEh4GTFo285m9UFe-T1mpMsAi_7R8V2gfibpX_SFLdLtBwf02_alQVsGA","token_type":"Bearer","expires_in":"3600"}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-10-08T11:23:03.7611666Z</x:t>
+  </x:si>
+  <x:si>
+    <x:t>0328c110-0422-40e8-91c1-f6a30ccbbf81</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{"MemberId":"9eb45736-827a-4751-9996-44088587006e","FirstName":"Arizona","LastName":"Rovicare ","UserName":"hospital@rovicare.com","EmailId":"hospital@rovicare.com","BusinessUnitId":"677920c1-831f-11ea-bd7d-04d9f5ab62dc","CompanyBusinessUnitId":"677920c1-831f-11ea-bd7d-04d9f5ab62dc","BusinessUnitName":"Arizona State Hospital","BusinessUnitType":"Provider","AssignedSettings":{"ReferralVisibilityInHrs":120,"ExtendedReferralVisibilityInHrs":192,"RatingReminderInDays":2,"ReferralViewDelayInMins":30,"IsEnableOrphanReferral":true,"IsEnable2StepAppointment":false,"AllowMemberAssigntoReferralForSendReferral":true,"AllowMemberViewAllReferralForSendReferral":true,"AllowMemberAssigntoReferralForReceiveReferral":false,"AllowMemberViewAllReferralForReceiveReferral":true,"DefaultHealthFacilityRating":2,"DefaultMedicareRating":4,"ReferralWithPatientPreferenceNote":null,"SearchAreaBy":"County","MaxSavedSearchAllowed":500,"IsContractSearched":false,"IsFaxReferralActive":true,"IsEmailReferralActive":true,"HadReferralWithAdvanceNotice":true,"WorkStartTime":null,"WorkEndTime":null,"MaxNumberOfOrganizationMembers":500,"MaxNumberOfImagesUploaded":10,"MaxSizeOfImagesUploadedInMB":50,"DurationOfHistoricalRecordsInDays":120,"LastSynOn":"2023-11-22T12:45:57.1111937Z","DefaultProviderType":null,"PatientVisibilityDays":30,"ConfirmReferralVisibilityInHrs":1.0,"LoginMethod":"Rovicare","DefaultFilter":"Medical","ShowInsurance":"Outgoing","IsTwelveTimeFormat":false,"ReceiveReferralDeliveryMode":"EFS","SendReferralToMemberViaFax":false,"EmrType":"Rovicare","EditRecordImportPatient":false,"AddRecordImportPatient":false,"OverrideRecordImportPatient":false,"AutomaticOverrideRecordImportPatient":true,"IsFullCapacity":true,"AcceptReferral":true,"IndicateToOrigin":true,"InpatientReferralActive":null,"OutpatientReferralActive":null,"PreAuthorizationRequired":false,"SharePatientRecord":false,"UpdateReferralResponse":true,"AutomaticallySharePatientRecord":false,"TentativeAcceptPatient":false,"ShowAverageResponseRate":true,"ResponseRateBusinessunitIds":"","DestinationCaseManagerConfig":"Email,Name,WorkNumber","CaseManagerDetailsConfig":"PhoneNumber,Email","DefaultShortlistPaginationCount":"50","DelayedClinicalRecordDays":null,"FaxNumberToSendCocDocument":null,"FollowUpRemovalTimeInMinutes":43200,"CocDocumentRequiringInsuranceList":[],"FollowUp7DayReminderTimeInMinute":10080,"FollowUp30DayReminderTimeInMinute":43200,"InpatientVisitReminderTimeInMinute":1440,"HiCommNotificationReminderInMinute":1440,"HiCommIPVDueDateOffsetDays":7,"CocDocumentReminderTimeInMinute":4320,"ShowAhcccsInfo":false,"UpdateCampus":false,"HiCommPatientReadmitIntervalInDays":30,"LocalTimeZoneId":null,"AssignPatientTagToHiCoM":null,"TeamAssignmentNotification":true,"WorkingDays":[],"Insurance":[],"CareRequirement":[],"ProviderType":[],"ServiceSetting":[],"SpecialProgram":[],"AgeGroup":[],"GenderType":[],"FacilityType":[],"AppointmentStatus":[],"FollowUpStatus":[],"DefaultRoute":null,"ConfigurableLogo":null,"Theme":null,"EnableDmeNotification":false,"WorkspaceConfigurations":[]},"DmeSettings":{"HcpNotificationMode":null,"EnableWoundCareQuantity":false,"EnableHhaCosmetics":false,"AllowShipToClinicianHome":false,"ShowEpisodeNumber":false},"EMRSetting":"{\"emrType\":\"Rovicare\",\"organizationName\":\"string\",\"organizationId\":\"string\",\"facilityId\":\"string\",\"AdvancedMdProgressNoteDateChanged\":\"string\",\"facilityUTCOffsetValue\":0.0,\"facilityAddress\":{\"streetAddress\":\"string\",\"city\":\"string\",\"state\":\"string\",\"zipcode\":\"string\"},\"providerType\":\"string\",\"facilityContact\":\"string\",\"healthCareResources\":{\"AllergyIntolerances\":true,\"Conditions\":true,\"Coverage\":true,\"DiagnosticReports\":true,\"Immunizations\":true,\"Medications\":true,\"ProgressNotes\":true,\"EmergencyContacts\":true,\"CarePlans\":true},\"MedicalRecordAccessLevel\":\"string\",\"HieFileInfo\":{\"BlobPathList\":[\"string\"],\"FileDirectoryFromUser\":\"string\",\"AddPatientIfNotExists\":true},\"siteId\":\"string\",\"fTPClientSettingModel\":{\"Host\":\"string\",\"Port\":0,\"UserName\":\"string\",\"Password\":\"string\",\"FileLocation\":\"string\",\"FileType\":\"string\"},\"EntityUpdates\":[{\"Entity\":\"string\",\"EntityLastUpdateTime\":\"2026-02-16T13:09:58.447Z\"}],\"EntityMetaData\":[{\"Entity\":\"string\",\"SearchParamters\":[{\"Key\":\"string\",\"Value\":\"string\"}]}]}","ServiceArea":"ZipCode","RoleName":"Organization Admin","HasAcceptedLicense":true,"AssignedFeatures":["NotificationFeature","ReceiveReferral","AppointmentDashboard","MobileApplication","SendReferral","ReceiveMedicalRecords","PreferredProviderList","Annotation","ShareCommandCenter","SurveyModule","CreateDMEOrder","ImportPatientByExcelsheet","SentReferralViaEmail","PendingServiceInitiationReminder","AddToPatientList","ShowCCRReport","GlobalChat","AdmitHistory","RecordReferral","PartialReferralConfirmation","AutoForwardChat","SentReferralViaFax","ShowReports","ShowCLRAReport","ReferralHistoryDashboard","AutomatedOriginStarRating","ShareReferrals","ShareMedicalRecords","LiveChat","PreferredProviderAvailability","CommandCenter","RecordReferralForOrigin","PendingReferralResponseReminder"],"BusinessUnitMemberId":"5b1a54d8-fd19-49f8-bb2e-fce04aa8b79e","PermissionList":["AcceptOrder","AddAppointment","AddAppointmentSlot","AddOrder","AddOrganization","AddOrganizationMember","AddPatient","AddPatientToCommandCenter","AddPreferredProvider","AddReferral","AddTag","AdminViewReports","AssignMember","AutoSyncOnAction","AutoSyncOnReferral","BulkActionForCommandCenter","CancelOrder","CancelReferral","CompulsaryServicesAndSpecialProgram","ConfirmPartialReferral","DeleteAppointment","DeleteAppointmentSlot","DeleteOrganizationMember","DeletePatient","DeletePreferredProvider","DeleteTag","DisableAutoConfirmReferral","DisableReferral","DisableReferralForServices","EditAppointment","EditAppointmentSlot","EditOrder","EditOrganization","EditOrganizationMember","EditPatient","EditPreferredProvider","EditReferral","EditTag","EnableMedicareRating","FaceSheetInMedicalRecords","GlobalChat","ImportPatientByCCDA","ImportPatientByExcelSheet","ImportPatientByFaceSheet","InsuranceProvider","LiveChat","ManageAllOrganization","ManageCompulsoryInsuranceForPatient","ManageCompulsoryServicesAndSpecialProgram","ManageOrganization","MemberAssignedToReferralForReceiveReferral","MessageBoard","MobileApplication","MovePatientToFollowUp","Notes","Notification","OnCallSupport","Order.Bulk.Download","Order.Bulk.Upload","Order.Bulk.View","Order.Document.Download","Order.Sign.Bypass","Order.Sign.OnBehalf","Order.Sign.Remind","Order.Workflow.Decline","Order.Workflow.Disposition","Order.Workflow.TakeOwnership","PatientPreference","PendingReferralsNotification","Prescriber.Search","ProvideRejectionReasonForReferral","ReceiveMedicalRecords","ReceiveReferral","ReceiveReferralSetting","ReferOrder","ReferralReport","ReferralTimeline","RejectOrder","RemovePatientFromCommandCenter","ResendReferral","ResponseReferral","ScheduleTransport","SendMedicalRecords","SendReferral","ShareCommandCenter","ShareMedicalRecords","ShareReferrals","ShareReferralsWithPreferredProviders","ShipOrder","ShowSpecialProgramNeeded","SuperAdmin","Track","UpdatePatientTask","UploadMedicalRecord","ViewAndManageCustomWorkspace","ViewAppointment","ViewAppointmentSlot","ViewMedicalRecord","ViewOrder","ViewOrganization","ViewOrganizationMember","ViewPatient","ViewPreferredProvider","ViewReferral","ViewReferralHistory","ViewTag"],"CacheId":"0328c110-0422-40e8-91c1-f6a30ccbbf81","AcceptedPolicyIds":[],"LoginError":[],"HasPowerBiReportAccess":false}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-10-08T11:23:04.7583115Z</x:t>
   </x:si>
   <x:si>
     <x:t>UserName</x:t>
@@ -283,13 +283,13 @@
     <x:t>hospital@rovicare.com</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-10-07T13:24:55.5538875Z</x:t>
+    <x:t>2026-10-08T11:23:04.8003583Z</x:t>
   </x:si>
   <x:si>
     <x:t>EmailId</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-10-07T13:24:55.5665513Z</x:t>
+    <x:t>2026-10-08T11:23:04.8213188Z</x:t>
   </x:si>
   <x:si>
     <x:t>BusinessUnitId</x:t>
@@ -298,13 +298,13 @@
     <x:t>677920c1-831f-11ea-bd7d-04d9f5ab62dc</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-10-07T13:24:55.5828710Z</x:t>
+    <x:t>2026-10-08T11:23:04.8385620Z</x:t>
   </x:si>
   <x:si>
     <x:t>CompanyBusinessUnitId</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-10-07T13:24:55.5959456Z</x:t>
+    <x:t>2026-10-08T11:23:04.8501362Z</x:t>
   </x:si>
   <x:si>
     <x:t>BusinessUnitMemberId</x:t>
@@ -313,7 +313,7 @@
     <x:t>5b1a54d8-fd19-49f8-bb2e-fce04aa8b79e</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-10-07T13:24:55.6103613Z</x:t>
+    <x:t>2026-10-08T11:23:04.8626560Z</x:t>
   </x:si>
   <x:si>
     <x:t>{"BusinessUnitId":"677920c1-831f-11ea-bd7d-04d9f5ab62dc","ParentBusinessUnitId":null,"CompanyType":"Not-for-Profit Corporation","OpenToNonContractedProvider":false,"Name":"Arizona State Hospital","Status":true,"Description":"Provide need &amp; clean environment Provide need ","LocationType":"ABHC/ACT","IsHeadOffice":null,"Latitude":"33.4297","Longitude":"-112.347611","BusinessUnitType":"Pacf","CreatedBy":null,"CreatedOn":null,"LastUpdatedBy":"fb715f93-8322-11ea-bd7d-04d9f5ab62dc","LastUpdatedOn":"2026-08-03T13:37:48.018548","WorkNumber":"2555555555","EmailId":"testingarizona@yopmail.com","Fax":"8069056421","BusinessUnitCategoryType":["Health Plan","Seriously Mentally Ill","care 1","DME Supplier","Telemedicine/Telehealth","Hospice","Mental Health","Home Health","Skilled Nursing(SNF)","ProviderTypeTest01","Residential Treatment Center","Transitional Housing","Outpatient Mental Health Services","DME Supplier","Transportation","Imaging Center","Psychiatry Providers","Behavioral Health Residential Facility","Attendant Care Provider","Acute Rehab","Social Determinants Of Health","Hospital Inpatient","Active Duty Military","Assistance With Activities Of Daily Living","Substance Use","Doctors And Clinicians","DME Provider","Emergency Mental Health Services"],"BusinessUnitAttributes":[{"EntityName":"AhcccsId","EntityValue":""}]}</x:t>
@@ -1840,16 +1840,16 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
+        <x:v>79</x:v>
+      </x:c>
+      <x:c r="C2" s="0" t="s">
+        <x:v>71</x:v>
+      </x:c>
+      <x:c r="D2" s="1" t="s">
+        <x:v>71</x:v>
+      </x:c>
+      <x:c r="E2" s="0" t="s">
         <x:v>70</x:v>
-      </x:c>
-      <x:c r="C2" s="0" t="s">
-        <x:v>71</x:v>
-      </x:c>
-      <x:c r="D2" s="1" t="s">
-        <x:v>71</x:v>
-      </x:c>
-      <x:c r="E2" s="0" t="s">
-        <x:v>72</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:5">
@@ -1857,33 +1857,33 @@
         <x:v>44</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
+        <x:v>72</x:v>
+      </x:c>
+      <x:c r="C3" s="0" t="s">
+        <x:v>71</x:v>
+      </x:c>
+      <x:c r="D3" s="1" t="s">
+        <x:v>71</x:v>
+      </x:c>
+      <x:c r="E3" s="0" t="s">
         <x:v>73</x:v>
-      </x:c>
-      <x:c r="C3" s="0" t="s">
-        <x:v>71</x:v>
-      </x:c>
-      <x:c r="D3" s="1" t="s">
-        <x:v>71</x:v>
-      </x:c>
-      <x:c r="E3" s="0" t="s">
-        <x:v>74</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:5" ht="143" customHeight="1">
       <x:c r="A4" s="0" t="s">
+        <x:v>74</x:v>
+      </x:c>
+      <x:c r="B4" s="0" t="s">
         <x:v>75</x:v>
       </x:c>
-      <x:c r="B4" s="0" t="s">
+      <x:c r="C4" s="0" t="s">
         <x:v>76</x:v>
       </x:c>
-      <x:c r="C4" s="0" t="s">
+      <x:c r="D4" s="1" t="s">
         <x:v>77</x:v>
       </x:c>
-      <x:c r="D4" s="1" t="s">
+      <x:c r="E4" s="0" t="s">
         <x:v>78</x:v>
-      </x:c>
-      <x:c r="E4" s="0" t="s">
-        <x:v>79</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:5" ht="409.5" customHeight="1">
@@ -1891,7 +1891,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B5" s="0" t="s">
-        <x:v>70</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="C5" s="0" t="s">
         <x:v>71</x:v>

</xml_diff>